<commit_message>
Update: 4/23-4/24交易数据 + OCR修复 + 图表优化
Changes:
- 新增4/23、4/24交易记录（两融+手机账户）
- 修复OCR解析：行间距阈值放宽、名称前后查找、去重机制
- 汇总报告：月度视图新增股票维度柱状图
- 个股图表改为上下排列，优化空间利用
- 饼图改进：亏损股票独立显示，标注盈/亏状态
</commit_message>
<xml_diff>
--- a/股票交易盈亏汇总.xlsx
+++ b/股票交易盈亏汇总.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1520,10 +1520,8 @@
           <t>手机账户</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>300502</t>
-        </is>
+      <c r="C22" s="2" t="n">
+        <v>300502</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
@@ -1571,10 +1569,8 @@
           <t>手机账户</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>688025</t>
-        </is>
+      <c r="C23" s="2" t="n">
+        <v>688025</v>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
@@ -1608,6 +1604,596 @@
       <c r="M23" s="2" t="inlineStr">
         <is>
           <t>1.39%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>两融账户</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>2594</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>比亚迪</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>100.16</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>99.98999999999999</v>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>10016</v>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>9999</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>-17</v>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>-0.17%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>两融账户</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>688041</v>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>海光信息</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>263.635</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>268.145</v>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>105454</v>
+      </c>
+      <c r="K25" s="2" t="n">
+        <v>107258</v>
+      </c>
+      <c r="L25" s="3" t="n">
+        <v>1804</v>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>1.71%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>两融账户</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>300394</v>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>天孚通信</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>369.015</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>351.03</v>
+      </c>
+      <c r="J26" s="2" t="n">
+        <v>73803</v>
+      </c>
+      <c r="K26" s="2" t="n">
+        <v>70206</v>
+      </c>
+      <c r="L26" s="4" t="n">
+        <v>-3597</v>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>-4.87%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>两融账户</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>300750</v>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>宁德时代</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>437.46</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>440.735</v>
+      </c>
+      <c r="J27" s="2" t="n">
+        <v>87492</v>
+      </c>
+      <c r="K27" s="2" t="n">
+        <v>88147</v>
+      </c>
+      <c r="L27" s="3" t="n">
+        <v>655</v>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>0.75%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>两融账户</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>688062</v>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>迈威生物</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>38.68</v>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>38.14</v>
+      </c>
+      <c r="J28" s="2" t="n">
+        <v>19340</v>
+      </c>
+      <c r="K28" s="2" t="n">
+        <v>19070</v>
+      </c>
+      <c r="L28" s="4" t="n">
+        <v>-270</v>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>-1.40%</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>手机账户</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>300750</v>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>宁德时代</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>436.75</v>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>442.85</v>
+      </c>
+      <c r="J29" s="2" t="n">
+        <v>43675</v>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>44285</v>
+      </c>
+      <c r="L29" s="3" t="n">
+        <v>610</v>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>1.40%</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>手机账户</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>300502</v>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>新易盛</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>602.91</v>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>610.5</v>
+      </c>
+      <c r="J30" s="2" t="n">
+        <v>60291</v>
+      </c>
+      <c r="K30" s="2" t="n">
+        <v>61050</v>
+      </c>
+      <c r="L30" s="3" t="n">
+        <v>759</v>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>1.26%</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>手机账户</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>300308</v>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>中际旭创</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>895.3099999999999</v>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>901.42</v>
+      </c>
+      <c r="J31" s="2" t="n">
+        <v>89531</v>
+      </c>
+      <c r="K31" s="2" t="n">
+        <v>90142</v>
+      </c>
+      <c r="L31" s="3" t="n">
+        <v>611</v>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>0.68%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>两融账户</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>688041</v>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>海光信息</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>900</v>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>900</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>278.6778</v>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>281.4227</v>
+      </c>
+      <c r="J32" s="2" t="n">
+        <v>250810</v>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>253280.45</v>
+      </c>
+      <c r="L32" s="3" t="n">
+        <v>2470.45</v>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>0.98%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>两融账户</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>688503</v>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>聚和材料</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>89.70999999999999</v>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>92.34</v>
+      </c>
+      <c r="J33" s="2" t="n">
+        <v>17942</v>
+      </c>
+      <c r="K33" s="2" t="n">
+        <v>18468</v>
+      </c>
+      <c r="L33" s="3" t="n">
+        <v>526</v>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>2.93%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>两融账户</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>300450</v>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>先导智能</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>55.94</v>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>57.23</v>
+      </c>
+      <c r="J34" s="2" t="n">
+        <v>11188</v>
+      </c>
+      <c r="K34" s="2" t="n">
+        <v>11446</v>
+      </c>
+      <c r="L34" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>2.31%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>手机账户</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>300502</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>新易盛</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>552.4299999999999</v>
+      </c>
+      <c r="I35" s="2" t="n">
+        <v>549.795</v>
+      </c>
+      <c r="J35" s="2" t="n">
+        <v>110486</v>
+      </c>
+      <c r="K35" s="2" t="n">
+        <v>109959</v>
+      </c>
+      <c r="L35" s="4" t="n">
+        <v>-527</v>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>-0.48%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: 2026-04-27 交易数据 + 报告更新
两融账户: +885.50 (海光+975, 天孚+172, 宁德-262)
手机账户: +124.00 (比亚迪+124)
当日合计: +1,009.50
</commit_message>
<xml_diff>
--- a/股票交易盈亏汇总.xlsx
+++ b/股票交易盈亏汇总.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M35"/>
+  <dimension ref="A1:M39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2157,10 +2157,8 @@
           <t>手机账户</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>300502</t>
-        </is>
+      <c r="C35" s="2" t="n">
+        <v>300502</v>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
@@ -2194,6 +2192,204 @@
       <c r="M35" s="2" t="inlineStr">
         <is>
           <t>-0.48%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>两融账户</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>300750</v>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>宁德时代</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>438</v>
+      </c>
+      <c r="I36" s="2" t="n">
+        <v>435.38</v>
+      </c>
+      <c r="J36" s="2" t="n">
+        <v>43800</v>
+      </c>
+      <c r="K36" s="2" t="n">
+        <v>43538</v>
+      </c>
+      <c r="L36" s="4" t="n">
+        <v>-262</v>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>-0.60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>两融账户</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>688041</v>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>海光信息</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>800</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>298.54</v>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>300.165</v>
+      </c>
+      <c r="J37" s="2" t="n">
+        <v>179124</v>
+      </c>
+      <c r="K37" s="2" t="n">
+        <v>180099</v>
+      </c>
+      <c r="L37" s="3" t="n">
+        <v>975</v>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>0.54%</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>两融账户</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>300394</v>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>天孚通信</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>323.31</v>
+      </c>
+      <c r="I38" s="2" t="n">
+        <v>325.035</v>
+      </c>
+      <c r="J38" s="2" t="n">
+        <v>32331</v>
+      </c>
+      <c r="K38" s="2" t="n">
+        <v>32503.5</v>
+      </c>
+      <c r="L38" s="3" t="n">
+        <v>172.5</v>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>0.53%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>手机账户</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>002594</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>比亚迪</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>102.56</v>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>103.18</v>
+      </c>
+      <c r="J39" s="2" t="n">
+        <v>20512</v>
+      </c>
+      <c r="K39" s="2" t="n">
+        <v>20636</v>
+      </c>
+      <c r="L39" s="3" t="n">
+        <v>124</v>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>0.60%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
分析 2026-04-30 两融+手机账户，盈亏 +561.65 +604.00 元
</commit_message>
<xml_diff>
--- a/股票交易盈亏汇总.xlsx
+++ b/股票交易盈亏汇总.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:M53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2791,46 +2791,293 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
+          <t>两融账户</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>688503</v>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>聚和材料</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>432</v>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>132</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>132</v>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>102.783</v>
+      </c>
+      <c r="I48" s="2" t="n">
+        <v>104</v>
+      </c>
+      <c r="J48" s="2" t="n">
+        <v>13567.35</v>
+      </c>
+      <c r="K48" s="2" t="n">
+        <v>13728</v>
+      </c>
+      <c r="L48" s="3" t="n">
+        <v>160.65</v>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>1.18%</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>两融账户</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>300054</v>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>鼎龙股份</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="H49" s="2" t="n">
+        <v>61.81</v>
+      </c>
+      <c r="I49" s="2" t="n">
+        <v>62.38</v>
+      </c>
+      <c r="J49" s="2" t="n">
+        <v>30905</v>
+      </c>
+      <c r="K49" s="2" t="n">
+        <v>31190</v>
+      </c>
+      <c r="L49" s="3" t="n">
+        <v>285</v>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>0.92%</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>两融账户</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>2222</v>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>福晶科技</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>87.42</v>
+      </c>
+      <c r="I50" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="J50" s="2" t="n">
+        <v>17484</v>
+      </c>
+      <c r="K50" s="2" t="n">
+        <v>17600</v>
+      </c>
+      <c r="L50" s="3" t="n">
+        <v>116</v>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>0.66%</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
           <t>平安账户</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>688778</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="C51" s="2" t="n">
+        <v>688778</v>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>厦钨新能源</t>
         </is>
       </c>
-      <c r="E48" s="2" t="n">
-        <v>200</v>
-      </c>
-      <c r="F48" s="2" t="n">
-        <v>200</v>
-      </c>
-      <c r="G48" s="2" t="n">
-        <v>200</v>
-      </c>
-      <c r="H48" s="2" t="n">
+      <c r="E51" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H51" s="2" t="n">
         <v>82.90000000000001</v>
       </c>
-      <c r="I48" s="2" t="n">
+      <c r="I51" s="2" t="n">
         <v>83.58</v>
       </c>
-      <c r="J48" s="2" t="n">
+      <c r="J51" s="2" t="n">
         <v>16580</v>
       </c>
-      <c r="K48" s="2" t="n">
+      <c r="K51" s="2" t="n">
         <v>16716</v>
       </c>
-      <c r="L48" s="3" t="n">
+      <c r="L51" s="3" t="n">
         <v>136</v>
       </c>
-      <c r="M48" s="2" t="inlineStr">
+      <c r="M51" s="2" t="inlineStr">
         <is>
           <t>0.82%</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>手机账户</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>002436</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>兴森科技</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="H52" s="2" t="n">
+        <v>27.22</v>
+      </c>
+      <c r="I52" s="2" t="n">
+        <v>27.78</v>
+      </c>
+      <c r="J52" s="2" t="n">
+        <v>13610</v>
+      </c>
+      <c r="K52" s="2" t="n">
+        <v>13890</v>
+      </c>
+      <c r="L52" s="3" t="n">
+        <v>280</v>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>2.06%</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>手机账户</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>301183</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>东田微</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H53" s="2" t="n">
+        <v>177</v>
+      </c>
+      <c r="I53" s="2" t="n">
+        <v>180.24</v>
+      </c>
+      <c r="J53" s="2" t="n">
+        <v>17700</v>
+      </c>
+      <c r="K53" s="2" t="n">
+        <v>18024</v>
+      </c>
+      <c r="L53" s="3" t="n">
+        <v>324</v>
+      </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>1.83%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
2026-06-01 交易分析：兴森科技+836.70 中际旭创+953.67 兴森科技(002436)+955.17 净盈利+2745.54
</commit_message>
<xml_diff>
--- a/股票交易盈亏汇总.xlsx
+++ b/股票交易盈亏汇总.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q192"/>
+  <dimension ref="A1:Q195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11971,10 +11971,8 @@
           <t>两融账户</t>
         </is>
       </c>
-      <c r="C189" s="2" t="inlineStr">
-        <is>
-          <t>688041</t>
-        </is>
+      <c r="C189" s="2" t="n">
+        <v>688041</v>
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
@@ -12034,10 +12032,8 @@
           <t>两融账户</t>
         </is>
       </c>
-      <c r="C190" s="2" t="inlineStr">
-        <is>
-          <t>688025</t>
-        </is>
+      <c r="C190" s="2" t="n">
+        <v>688025</v>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
@@ -12097,10 +12093,8 @@
           <t>两融账户</t>
         </is>
       </c>
-      <c r="C191" s="2" t="inlineStr">
-        <is>
-          <t>688035</t>
-        </is>
+      <c r="C191" s="2" t="n">
+        <v>688035</v>
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
@@ -12160,10 +12154,8 @@
           <t>两融账户</t>
         </is>
       </c>
-      <c r="C192" s="2" t="inlineStr">
-        <is>
-          <t>002222</t>
-        </is>
+      <c r="C192" s="2" t="n">
+        <v>2222</v>
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
@@ -12209,6 +12201,195 @@
       <c r="Q192" s="2" t="inlineStr">
         <is>
           <t>⚠️仅卖出未平仓</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t>手机账户</t>
+        </is>
+      </c>
+      <c r="C193" s="2" t="inlineStr">
+        <is>
+          <t>688503</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>聚和材料</t>
+        </is>
+      </c>
+      <c r="E193" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="F193" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G193" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H193" s="2" t="n">
+        <v>88.76000000000001</v>
+      </c>
+      <c r="I193" s="2" t="n">
+        <v>93.04000000000001</v>
+      </c>
+      <c r="J193" s="2" t="n">
+        <v>17752</v>
+      </c>
+      <c r="K193" s="2" t="n">
+        <v>18608</v>
+      </c>
+      <c r="L193" s="3" t="n">
+        <v>856</v>
+      </c>
+      <c r="M193" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="N193" s="2" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="O193" s="2" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="P193" s="3" t="n">
+        <v>836.7</v>
+      </c>
+      <c r="Q193" s="2" t="inlineStr">
+        <is>
+          <t>4.71%</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>手机账户</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr">
+        <is>
+          <t>300308</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>中际旭创</t>
+        </is>
+      </c>
+      <c r="E194" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F194" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G194" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H194" s="2" t="n">
+        <v>1138.65</v>
+      </c>
+      <c r="I194" s="2" t="n">
+        <v>1148.99</v>
+      </c>
+      <c r="J194" s="2" t="n">
+        <v>113865</v>
+      </c>
+      <c r="K194" s="2" t="n">
+        <v>114899</v>
+      </c>
+      <c r="L194" s="3" t="n">
+        <v>1034</v>
+      </c>
+      <c r="M194" s="2" t="n">
+        <v>22.88</v>
+      </c>
+      <c r="N194" s="2" t="n">
+        <v>57.45</v>
+      </c>
+      <c r="O194" s="2" t="n">
+        <v>80.33</v>
+      </c>
+      <c r="P194" s="3" t="n">
+        <v>953.67</v>
+      </c>
+      <c r="Q194" s="2" t="inlineStr">
+        <is>
+          <t>0.84%</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B195" s="2" t="inlineStr">
+        <is>
+          <t>手机账户</t>
+        </is>
+      </c>
+      <c r="C195" s="2" t="inlineStr">
+        <is>
+          <t>002436</t>
+        </is>
+      </c>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>兴森科技</t>
+        </is>
+      </c>
+      <c r="E195" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F195" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G195" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H195" s="2" t="n">
+        <v>38.67</v>
+      </c>
+      <c r="I195" s="2" t="n">
+        <v>39.655</v>
+      </c>
+      <c r="J195" s="2" t="n">
+        <v>38670</v>
+      </c>
+      <c r="K195" s="2" t="n">
+        <v>39655</v>
+      </c>
+      <c r="L195" s="3" t="n">
+        <v>985</v>
+      </c>
+      <c r="M195" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="N195" s="2" t="n">
+        <v>19.83</v>
+      </c>
+      <c r="O195" s="2" t="n">
+        <v>29.83</v>
+      </c>
+      <c r="P195" s="3" t="n">
+        <v>955.17</v>
+      </c>
+      <c r="Q195" s="2" t="inlineStr">
+        <is>
+          <t>2.47%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
2026-07-08 双账户分析：海光+4594 天孚+452 澜起+449 净盈利+5411.46
</commit_message>
<xml_diff>
--- a/股票交易盈亏汇总.xlsx
+++ b/股票交易盈亏汇总.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q397"/>
+  <dimension ref="A1:Q401"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24537,10 +24537,8 @@
           <t>两融账户+手机账户</t>
         </is>
       </c>
-      <c r="C395" s="2" t="inlineStr">
-        <is>
-          <t>300502</t>
-        </is>
+      <c r="C395" s="2" t="n">
+        <v>300502</v>
       </c>
       <c r="D395" s="2" t="inlineStr">
         <is>
@@ -24600,10 +24598,8 @@
           <t>两融账户+手机账户</t>
         </is>
       </c>
-      <c r="C396" s="2" t="inlineStr">
-        <is>
-          <t>688008</t>
-        </is>
+      <c r="C396" s="2" t="n">
+        <v>688008</v>
       </c>
       <c r="D396" s="2" t="inlineStr">
         <is>
@@ -24663,10 +24659,8 @@
           <t>两融账户+手机账户</t>
         </is>
       </c>
-      <c r="C397" s="2" t="inlineStr">
-        <is>
-          <t>688041</t>
-        </is>
+      <c r="C397" s="2" t="n">
+        <v>688041</v>
       </c>
       <c r="D397" s="2" t="inlineStr">
         <is>
@@ -24712,6 +24706,258 @@
       <c r="Q397" s="2" t="inlineStr">
         <is>
           <t>0.82%</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B398" s="2" t="inlineStr">
+        <is>
+          <t>两融账户+手机账户</t>
+        </is>
+      </c>
+      <c r="C398" s="2" t="inlineStr">
+        <is>
+          <t>688008</t>
+        </is>
+      </c>
+      <c r="D398" s="2" t="inlineStr">
+        <is>
+          <t>澜起科技</t>
+        </is>
+      </c>
+      <c r="E398" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="F398" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="G398" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="H398" s="2" t="n">
+        <v>251.135</v>
+      </c>
+      <c r="I398" s="2" t="n">
+        <v>252.435</v>
+      </c>
+      <c r="J398" s="2" t="n">
+        <v>100454</v>
+      </c>
+      <c r="K398" s="2" t="n">
+        <v>100974</v>
+      </c>
+      <c r="L398" s="3" t="n">
+        <v>520</v>
+      </c>
+      <c r="M398" s="2" t="n">
+        <v>20.14</v>
+      </c>
+      <c r="N398" s="2" t="n">
+        <v>50.49</v>
+      </c>
+      <c r="O398" s="2" t="n">
+        <v>70.63</v>
+      </c>
+      <c r="P398" s="3" t="n">
+        <v>449.37</v>
+      </c>
+      <c r="Q398" s="2" t="inlineStr">
+        <is>
+          <t>0.45%</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B399" s="2" t="inlineStr">
+        <is>
+          <t>两融账户+手机账户</t>
+        </is>
+      </c>
+      <c r="C399" s="2" t="inlineStr">
+        <is>
+          <t>688041</t>
+        </is>
+      </c>
+      <c r="D399" s="2" t="inlineStr">
+        <is>
+          <t>海光信息</t>
+        </is>
+      </c>
+      <c r="E399" s="2" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F399" s="2" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G399" s="2" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H399" s="2" t="n">
+        <v>345.5621</v>
+      </c>
+      <c r="I399" s="2" t="n">
+        <v>349.0878</v>
+      </c>
+      <c r="J399" s="2" t="n">
+        <v>483786.96</v>
+      </c>
+      <c r="K399" s="2" t="n">
+        <v>488722.89</v>
+      </c>
+      <c r="L399" s="3" t="n">
+        <v>4935.93</v>
+      </c>
+      <c r="M399" s="2" t="n">
+        <v>97.25</v>
+      </c>
+      <c r="N399" s="2" t="n">
+        <v>244.36</v>
+      </c>
+      <c r="O399" s="2" t="n">
+        <v>341.61</v>
+      </c>
+      <c r="P399" s="3" t="n">
+        <v>4594.32</v>
+      </c>
+      <c r="Q399" s="2" t="inlineStr">
+        <is>
+          <t>0.95%</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B400" s="2" t="inlineStr">
+        <is>
+          <t>两融账户+手机账户</t>
+        </is>
+      </c>
+      <c r="C400" s="2" t="inlineStr">
+        <is>
+          <t>688041</t>
+        </is>
+      </c>
+      <c r="D400" s="2" t="inlineStr">
+        <is>
+          <t>海光信息</t>
+        </is>
+      </c>
+      <c r="E400" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F400" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="G400" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H400" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I400" s="2" t="n">
+        <v>349.0878</v>
+      </c>
+      <c r="J400" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K400" s="2" t="n">
+        <v>139635.11</v>
+      </c>
+      <c r="L400" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M400" s="2" t="n">
+        <v>13.96</v>
+      </c>
+      <c r="N400" s="2" t="n">
+        <v>69.81999999999999</v>
+      </c>
+      <c r="O400" s="2" t="n">
+        <v>83.78</v>
+      </c>
+      <c r="P400" s="4" t="n">
+        <v>-83.78</v>
+      </c>
+      <c r="Q400" s="2" t="inlineStr">
+        <is>
+          <t>⚠️多卖未平仓</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B401" s="2" t="inlineStr">
+        <is>
+          <t>两融账户+手机账户</t>
+        </is>
+      </c>
+      <c r="C401" s="2" t="inlineStr">
+        <is>
+          <t>300394</t>
+        </is>
+      </c>
+      <c r="D401" s="2" t="inlineStr">
+        <is>
+          <t>天孚通信</t>
+        </is>
+      </c>
+      <c r="E401" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F401" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G401" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H401" s="2" t="n">
+        <v>244.24</v>
+      </c>
+      <c r="I401" s="2" t="n">
+        <v>248.98</v>
+      </c>
+      <c r="J401" s="2" t="n">
+        <v>24424</v>
+      </c>
+      <c r="K401" s="2" t="n">
+        <v>24898</v>
+      </c>
+      <c r="L401" s="3" t="n">
+        <v>474</v>
+      </c>
+      <c r="M401" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="N401" s="2" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="O401" s="2" t="n">
+        <v>22.45</v>
+      </c>
+      <c r="P401" s="3" t="n">
+        <v>451.55</v>
+      </c>
+      <c r="Q401" s="2" t="inlineStr">
+        <is>
+          <t>1.85%</t>
         </is>
       </c>
     </row>

</xml_diff>